<commit_message>
Added CDFs to Model
CDFs still not connected to uncertainty. Not sure how to yet
</commit_message>
<xml_diff>
--- a/Battery_Capacity/Battery_Capacity.xlsx
+++ b/Battery_Capacity/Battery_Capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07531a99d7244c5b/Documents/GitHub/ASE6002PEK/Battery_Capacity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18173" documentId="114_{C6D45846-3148-4081-A19D-15A1F6BD3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F309C7A4-76F3-45CE-9884-A1CC66448F22}"/>
+  <xr:revisionPtr revIDLastSave="20489" documentId="114_{C6D45846-3148-4081-A19D-15A1F6BD3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4B9C968-C8D4-4F22-B316-18D24618117B}"/>
   <bookViews>
     <workbookView xWindow="9105" yWindow="5325" windowWidth="38700" windowHeight="15345" xr2:uid="{21964307-0BB7-4DE0-BD23-E82C9EC81DDB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <definedName name="UNC_Batt_Cap">Sheet1!$B$9</definedName>
     <definedName name="UNC_Batt_Cost">Sheet1!$B$10</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -518,7 +518,7 @@
       </c>
       <c r="B5">
         <f>Pack_Count*5*11.1*3600*UNC_Batt_Cap</f>
-        <v>583906.56954386272</v>
+        <v>544264.60667248687</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -545,7 +545,7 @@
       </c>
       <c r="B7">
         <f>3.15*3*B3*B10</f>
-        <v>29.069588798896493</v>
+        <v>28.699178325505883</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -553,7 +553,7 @@
         <v>12</v>
       </c>
       <c r="B9">
-        <v>0.97415176767411205</v>
+        <v>0.90801569348095901</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -564,7 +564,7 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>1.0253823209487301</v>
+        <v>1.01231669578504</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Updated model to connect CDFs
</commit_message>
<xml_diff>
--- a/Battery_Capacity/Battery_Capacity.xlsx
+++ b/Battery_Capacity/Battery_Capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07531a99d7244c5b/Documents/GitHub/ASE6002PEK/Battery_Capacity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20489" documentId="114_{C6D45846-3148-4081-A19D-15A1F6BD3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4B9C968-C8D4-4F22-B316-18D24618117B}"/>
+  <xr:revisionPtr revIDLastSave="20579" documentId="114_{C6D45846-3148-4081-A19D-15A1F6BD3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF4A5745-F50D-4744-A74B-D6E6D7F4855D}"/>
   <bookViews>
     <workbookView xWindow="9105" yWindow="5325" windowWidth="38700" windowHeight="15345" xr2:uid="{21964307-0BB7-4DE0-BD23-E82C9EC81DDB}"/>
   </bookViews>
@@ -518,7 +518,7 @@
       </c>
       <c r="B5">
         <f>Pack_Count*5*11.1*3600*UNC_Batt_Cap</f>
-        <v>544264.60667248687</v>
+        <v>59084.818422765769</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -545,7 +545,7 @@
       </c>
       <c r="B7">
         <f>3.15*3*B3*B10</f>
-        <v>28.699178325505883</v>
+        <v>3.0735752822820297</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -553,7 +553,7 @@
         <v>12</v>
       </c>
       <c r="B9">
-        <v>0.90801569348095901</v>
+        <v>9.8573270641918204E-2</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -564,7 +564,7 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>1.01231669578504</v>
+        <v>0.10841535387238201</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Added Trade Study for Task 5
</commit_message>
<xml_diff>
--- a/Battery_Capacity/Battery_Capacity.xlsx
+++ b/Battery_Capacity/Battery_Capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/07531a99d7244c5b/Documents/GitHub/ASE6002PEK/Battery_Capacity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21551" documentId="114_{C6D45846-3148-4081-A19D-15A1F6BD3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF3D7E91-4C46-4895-8FFB-1B5EFB644867}"/>
+  <xr:revisionPtr revIDLastSave="24551" documentId="114_{C6D45846-3148-4081-A19D-15A1F6BD3370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CC2BB63-0D24-4EB5-86DC-6C7E32D1172B}"/>
   <bookViews>
     <workbookView xWindow="9105" yWindow="5325" windowWidth="38700" windowHeight="15345" xr2:uid="{21964307-0BB7-4DE0-BD23-E82C9EC81DDB}"/>
   </bookViews>
@@ -518,7 +518,7 @@
       </c>
       <c r="B5">
         <f>Pack_Count*5*11.1*3600*UNC_Batt_Cap</f>
-        <v>58273.0977554118</v>
+        <v>63149.991064902228</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -545,7 +545,7 @@
       </c>
       <c r="B7">
         <f>3.15*3*B3*B10</f>
-        <v>3.4863179451803732</v>
+        <v>25.000673015324427</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -553,7 +553,7 @@
         <v>12</v>
       </c>
       <c r="B9">
-        <v>9.7219048640993996E-2</v>
+        <v>0.10535534044861899</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -564,7 +564,7 @@
         <v>14</v>
       </c>
       <c r="B10">
-        <v>0.122974177960507</v>
+        <v>0.88185795468516504</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>

</xml_diff>